<commit_message>
import HSPK Detail v0
</commit_message>
<xml_diff>
--- a/resources/template/Template Isian SSH.xlsx
+++ b/resources/template/Template Isian SSH.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\kab_bogor\resources\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Downloads\kabbogor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5333EB3-4622-405D-84EC-ED13B4EF6001}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA0D91E-7680-440C-AED4-8679B91915DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{55E3F4EF-3A0D-4D89-A79F-0AF6D60BB7D9}"/>
   </bookViews>
@@ -20,18 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="35">
   <si>
     <t>IdKelBrg</t>
   </si>
@@ -63,74 +57,109 @@
     <t>Harga</t>
   </si>
   <si>
-    <t>A001</t>
-  </si>
-  <si>
-    <t>Kaca</t>
-  </si>
-  <si>
-    <t>SBU</t>
-  </si>
-  <si>
     <t>01</t>
   </si>
   <si>
-    <t>Kaca Bening</t>
-  </si>
-  <si>
-    <t>Kaca Bening Tebal 3mm</t>
-  </si>
-  <si>
-    <t>m2</t>
+    <t>Batu</t>
+  </si>
+  <si>
+    <t>Buah</t>
+  </si>
+  <si>
+    <t>1.1.7.01.01.01.005</t>
+  </si>
+  <si>
+    <t>SSH</t>
+  </si>
+  <si>
+    <t>Pinggir beton 10 x 20 x 35</t>
+  </si>
+  <si>
+    <t>Pinggir beton 15 x 35 x 50 K-225</t>
   </si>
   <si>
     <t>02</t>
   </si>
   <si>
-    <t>Kaca Bening Tebal 5mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kaca Tempered </t>
-  </si>
-  <si>
-    <t>Kaca Tempered  Tebal 3mm</t>
-  </si>
-  <si>
-    <t>A002</t>
-  </si>
-  <si>
-    <t>Batu</t>
-  </si>
-  <si>
-    <t>Batu Bata Merah</t>
-  </si>
-  <si>
-    <t>Batu Bata Merah 17 x 8 x 4cm</t>
-  </si>
-  <si>
-    <t>Batu Bata Kapur Putih</t>
-  </si>
-  <si>
-    <t>Batu Bata Ringan Hebel</t>
-  </si>
-  <si>
-    <t>m3</t>
-  </si>
-  <si>
-    <t>Buah</t>
+    <t>03</t>
+  </si>
+  <si>
+    <t>Bara</t>
+  </si>
+  <si>
+    <t>Kg</t>
+  </si>
+  <si>
+    <t>M3</t>
+  </si>
+  <si>
+    <t>1.1.7.01.01.01.002</t>
+  </si>
+  <si>
+    <t>Semen</t>
+  </si>
+  <si>
+    <t>Bahan adukan mortar</t>
+  </si>
+  <si>
+    <t>Bahan grouting</t>
+  </si>
+  <si>
+    <t>Semen Instan</t>
+  </si>
+  <si>
+    <t>Acian diatas beton dan plester AM86 40 kg</t>
+  </si>
+  <si>
+    <t>Zak</t>
+  </si>
+  <si>
+    <t>1.1.7.01.01.05.002</t>
+  </si>
+  <si>
+    <t>Kayu</t>
+  </si>
+  <si>
+    <t>Kayu Kaso</t>
+  </si>
+  <si>
+    <t>Ukuran 5/7 cm</t>
+  </si>
+  <si>
+    <t>Batang</t>
+  </si>
+  <si>
+    <t>Kayu kaso 5/7 kelas III</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -156,16 +185,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{F09928A5-97F7-4CD5-A3AB-51020F12F0BF}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -478,19 +514,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54B9473C-5850-4A4E-971E-9610A1BECAC3}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.85546875" customWidth="1"/>
     <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -526,326 +562,487 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>10</v>
+      <c r="A2" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I2">
-        <v>2022</v>
-      </c>
-      <c r="J2">
-        <v>85000</v>
+        <v>2025</v>
+      </c>
+      <c r="J2" s="3">
+        <v>37400</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
+      <c r="A3" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I3">
-        <v>2023</v>
-      </c>
-      <c r="J3">
-        <v>90000</v>
+        <v>2026</v>
+      </c>
+      <c r="J3" s="3">
+        <v>38500</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
+      <c r="A4" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I4">
-        <v>2022</v>
-      </c>
-      <c r="J4">
-        <v>90000</v>
+        <v>2025</v>
+      </c>
+      <c r="J4" s="3">
+        <v>112000</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
+      <c r="A5" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5">
+        <v>2026</v>
+      </c>
+      <c r="J5" s="3">
+        <v>115100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5">
-        <v>2023</v>
-      </c>
-      <c r="J5">
-        <v>97500</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6">
+        <v>2025</v>
+      </c>
+      <c r="J6" s="3">
+        <v>339200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G6" t="s">
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" t="s">
         <v>20</v>
       </c>
-      <c r="H6" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6">
-        <v>2022</v>
-      </c>
-      <c r="J6">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" t="s">
-        <v>16</v>
-      </c>
       <c r="I7">
-        <v>2023</v>
-      </c>
-      <c r="J7">
-        <v>210000</v>
+        <v>2026</v>
+      </c>
+      <c r="J7" s="3">
+        <v>376100</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>21</v>
+      <c r="A8" t="s">
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E8" t="s">
         <v>23</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>24</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="I8">
-        <v>2022</v>
-      </c>
-      <c r="J8">
-        <v>600</v>
+        <v>2025</v>
+      </c>
+      <c r="J8" s="3">
+        <v>986200</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>21</v>
+      <c r="A9" t="s">
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E9" t="s">
         <v>23</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>24</v>
       </c>
       <c r="H9" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="I9">
-        <v>2023</v>
-      </c>
-      <c r="J9">
-        <v>650</v>
+        <v>2026</v>
+      </c>
+      <c r="J9" s="3">
+        <v>1003600</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>21</v>
+      <c r="A10" t="s">
+        <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" t="s">
-        <v>26</v>
-      </c>
       <c r="H10" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="I10">
-        <v>2022</v>
-      </c>
-      <c r="J10">
-        <v>700000</v>
+        <v>2025</v>
+      </c>
+      <c r="J10" s="3">
+        <v>22300</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>21</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11">
+        <v>2026</v>
+      </c>
+      <c r="J11" s="3">
+        <v>24700</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" t="s">
         <v>26</v>
       </c>
-      <c r="H11" t="s">
+      <c r="F12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" t="s">
         <v>27</v>
       </c>
-      <c r="I11">
-        <v>2023</v>
-      </c>
-      <c r="J11">
-        <v>730000</v>
+      <c r="H12" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12">
+        <v>2025</v>
+      </c>
+      <c r="J12" s="3">
+        <v>220200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13">
+        <v>2026</v>
+      </c>
+      <c r="J13" s="3">
+        <v>226200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" t="s">
+        <v>32</v>
+      </c>
+      <c r="H14" t="s">
+        <v>33</v>
+      </c>
+      <c r="I14">
+        <v>2025</v>
+      </c>
+      <c r="J14" s="3">
+        <v>62700</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
+        <v>32</v>
+      </c>
+      <c r="H15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15">
+        <v>2026</v>
+      </c>
+      <c r="J15" s="3">
+        <v>70200</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16">
+        <v>2026</v>
+      </c>
+      <c r="J16" s="3">
+        <v>1826100</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>